<commit_message>
Move invoice/receipt title to top-center, enlarge it
- Templates: title (ใบแจ้งหนี้/ใบส่งสินค้า, ใบเสร็จรับเงิน) was in J3/J4
  right-aligned next to the org name. Moved into the previously-blank
  A1:K1/A2:K2 rows, merged full-width, centered, font bumped
  16→24 / 14→16.
- fill_invoice.py: receipt ต้นฉบับ/คู่ฉบับ override now writes to
  A1/A2 instead of the old J3/J4.
- Verified via synthetic data through the real pipeline (fill_invoice
  -> xlsx_to_pdf.ps1 -> pdfplumber render) for invoice, receipt
  original, and receipt copy pages — centered, larger, no overflow.
</commit_message>
<xml_diff>
--- a/server/templates/receipt-template.xlsx
+++ b/server/templates/receipt-template.xlsx
@@ -30,7 +30,7 @@
     <numFmt numFmtId="170" formatCode="#,##0;\-#,##0;&quot;&quot;"/>
     <numFmt numFmtId="171" formatCode="0\ &quot; EA&quot;"/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <charset val="222"/>
@@ -182,6 +182,16 @@
       <color theme="1"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Cordia New"/>
+      <b val="1"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Cordia New"/>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -239,7 +249,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="55">
+  <borders count="57">
     <border>
       <left/>
       <right/>
@@ -873,13 +883,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="202">
+  <cellXfs count="207">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1320,6 +1354,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="55" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="56" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1729,22 +1772,30 @@
     <col width="8.7265625" customWidth="1" style="48" min="15" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="53" t="n"/>
-      <c r="B1" s="54" t="n"/>
-      <c r="C1" s="54" t="n"/>
-      <c r="D1" s="54" t="n"/>
-      <c r="E1" s="54" t="n"/>
-      <c r="F1" s="54" t="n"/>
-      <c r="G1" s="54" t="n"/>
-      <c r="H1" s="54" t="n"/>
-      <c r="I1" s="54" t="n"/>
-      <c r="J1" s="54" t="n"/>
-      <c r="K1" s="55" t="n"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="56" t="n"/>
-      <c r="K2" s="57" t="n"/>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="202" t="inlineStr">
+        <is>
+          <t>ใบเสร็จรับเงิน</t>
+        </is>
+      </c>
+      <c r="B1" s="203" t="n"/>
+      <c r="C1" s="203" t="n"/>
+      <c r="D1" s="203" t="n"/>
+      <c r="E1" s="203" t="n"/>
+      <c r="F1" s="203" t="n"/>
+      <c r="G1" s="203" t="n"/>
+      <c r="H1" s="203" t="n"/>
+      <c r="I1" s="203" t="n"/>
+      <c r="J1" s="203" t="n"/>
+      <c r="K1" s="204" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="205" t="inlineStr">
+        <is>
+          <t>RECEIPT</t>
+        </is>
+      </c>
+      <c r="K2" s="206" t="n"/>
     </row>
     <row r="3" ht="23.5" customHeight="1">
       <c r="A3" s="56" t="n"/>
@@ -1760,11 +1811,7 @@
       <c r="G3" s="60" t="n"/>
       <c r="H3" s="60" t="n"/>
       <c r="I3" s="60" t="n"/>
-      <c r="J3" s="35" t="inlineStr">
-        <is>
-          <t>ใบเสร็จรับเงิน</t>
-        </is>
-      </c>
+      <c r="J3" s="35" t="n"/>
       <c r="K3" s="57" t="n"/>
       <c r="M3" s="36" t="n"/>
     </row>
@@ -1782,11 +1829,7 @@
       <c r="G4" s="60" t="n"/>
       <c r="H4" s="60" t="n"/>
       <c r="I4" s="62" t="n"/>
-      <c r="J4" s="37" t="inlineStr">
-        <is>
-          <t>RECEIPT</t>
-        </is>
-      </c>
+      <c r="J4" s="37" t="n"/>
       <c r="K4" s="57" t="n"/>
       <c r="M4" s="38" t="inlineStr">
         <is>
@@ -2914,25 +2957,27 @@
       <c r="L52" s="47" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="E24:G24"/>
+  <mergeCells count="20">
     <mergeCell ref="E28:G28"/>
-    <mergeCell ref="E22:G22"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="J9:J10"/>
+    <mergeCell ref="A1:K1"/>
     <mergeCell ref="E27:G27"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="E24:G24"/>
     <mergeCell ref="E23:G23"/>
     <mergeCell ref="E17:G17"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="J31:J32"/>
     <mergeCell ref="E29:G29"/>
     <mergeCell ref="J39:J40"/>
-    <mergeCell ref="E25:G25"/>
     <mergeCell ref="E20:G20"/>
-    <mergeCell ref="E16:G16"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2362204724409449" right="0.2362204724409449" top="0.7480314960629921" bottom="0.7480314960629921" header="0.3937007874015748" footer="0.3149606299212598"/>

</xml_diff>